<commit_message>
Polish repo for public release
Rewrite README with badges, quick-start install instructions, and a
disclaimer covering third-party mod licensing. Add MIT license for the
documentation/packaging content (does not cover bundled mod jars).
Remove fixed player-count references across docs and spreadsheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/minecraft_26_2_neoforge_mod_deployment.xlsx
+++ b/minecraft_26_2_neoforge_mod_deployment.xlsx
@@ -657,18 +657,6 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Expected Players</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-    </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -810,7 +798,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Reasonable for a 5-player private co-op server, but no longer lightweight</t>
+          <t>Reasonable for a private co-op server, but no longer lightweight</t>
         </is>
       </c>
     </row>
@@ -1500,18 +1488,6 @@
       <c r="B8" s="5" t="inlineStr">
         <is>
           <t>4 GB</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Expected players</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
         </is>
       </c>
     </row>

</xml_diff>